<commit_message>
updated new product list
</commit_message>
<xml_diff>
--- a/docs/Defect_Tracker Template_v0.1.xlsx
+++ b/docs/Defect_Tracker Template_v0.1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3d79fe2bc3d7eff9/Desktop/AI_Ecommerce_project/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="514" documentId="13_ncr:101_{A9B59A9A-789B-4A89-A90D-BB9A1B756E8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{73CE82B6-2C78-481C-B704-7E737218987E}"/>
+  <xr:revisionPtr revIDLastSave="516" documentId="13_ncr:101_{A9B59A9A-789B-4A89-A90D-BB9A1B756E8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8F950A6F-5EC9-40C8-BBD9-3C30430086A1}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -416,6 +416,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -705,6 +709,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:K20"/>
   <sheetFormatPr defaultColWidth="17.54296875" defaultRowHeight="21" x14ac:dyDescent="0.5"/>
   <cols>
@@ -722,7 +729,7 @@
     <col min="12" max="16384" width="17.54296875" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="2" customFormat="1" ht="42" x14ac:dyDescent="0.5">
+    <row r="1" spans="1:11" s="2" customFormat="1" ht="63" x14ac:dyDescent="0.5">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -764,9 +771,7 @@
       <c r="B2" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="10">
-        <v>46030</v>
-      </c>
+      <c r="C2" s="10"/>
       <c r="D2" s="11" t="s">
         <v>21</v>
       </c>
@@ -967,7 +972,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="84" x14ac:dyDescent="0.5">
+    <row r="8" spans="1:11" ht="63" x14ac:dyDescent="0.5">
       <c r="A8" s="8">
         <v>7</v>
       </c>
@@ -1002,7 +1007,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="84" x14ac:dyDescent="0.5">
+    <row r="9" spans="1:11" ht="63" x14ac:dyDescent="0.5">
       <c r="A9" s="16">
         <v>8</v>
       </c>
@@ -1271,7 +1276,7 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" horizontalDpi="200" verticalDpi="200" r:id="rId1"/>
+  <pageSetup scale="38" orientation="portrait" horizontalDpi="200" verticalDpi="200" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -1457,18 +1462,18 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1490,18 +1495,25 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B149665-BEBB-4C97-BAA6-72374EAA67F9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="b67b99c0-208c-4860-83e0-51466af787c4"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{20D196DE-5AC8-4D3B-8CD7-1A2AE6EEDD72}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8B149665-BEBB-4C97-BAA6-72374EAA67F9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>